<commit_message>
Remove board-approval wording from PDFs, dashboards and workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017mGL574Juds5KRyHsEvAPk
</commit_message>
<xml_diff>
--- a/waqf-2026/محفظة-الوقف-2026.xlsx
+++ b/waqf-2026/محفظة-الوقف-2026.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="447">
   <si>
-    <t xml:space="preserve">المحفظة المعتمدة من مجلس الإدارة — 1,500,000 ريال</t>
+    <t xml:space="preserve">المحفظة المعتمدة — 1,500,000 ريال</t>
   </si>
   <si>
     <t xml:space="preserve">الأسعار: آخر إغلاق على أرقام في 11–12 أكتوبر 2026 · الخلايا الزرقاء مدخلات قابلة للتعديل وتعيد حساب كل شيء تلقائياً</t>
@@ -341,7 +341,7 @@
     <t xml:space="preserve">مستبعد</t>
   </si>
   <si>
-    <t xml:space="preserve">استُبعد بقرار مجلس الإدارة (أكتوبر 2026)</t>
+    <t xml:space="preserve">نمو بطيء وتراجع السعر 16% خلال 6 أشهر</t>
   </si>
   <si>
     <t xml:space="preserve">بنك الجزيرة</t>
@@ -629,6 +629,9 @@
     <t xml:space="preserve">~100%</t>
   </si>
   <si>
+    <t xml:space="preserve">يوزع ~100% من أرباحه دون هامش أمان</t>
+  </si>
+  <si>
     <t xml:space="preserve">بوبا العربية</t>
   </si>
   <si>
@@ -809,10 +812,10 @@
     <t xml:space="preserve">ملاحظات</t>
   </si>
   <si>
-    <t xml:space="preserve">اعتماد سياسة الاستثمار والتوزيع (الورقة: سياسة الوقف) من الناظر ومجلس الجمعية</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ناظر الوقف / مجلس الجمعية</t>
+    <t xml:space="preserve">اعتماد سياسة الاستثمار والتوزيع (الورقة: سياسة الوقف) من ناظر الوقف</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ناظر الوقف</t>
   </si>
   <si>
     <t xml:space="preserve">لم يبدأ</t>
@@ -851,9 +854,6 @@
     <t xml:space="preserve">توثيق/تسجيل الوقف لدى الهيئة العامة للأوقاف وإرفاق كشف المحفظة</t>
   </si>
   <si>
-    <t xml:space="preserve">ناظر الوقف</t>
-  </si>
-  <si>
     <t xml:space="preserve">شهادة تسجيل</t>
   </si>
   <si>
@@ -1049,7 +1049,7 @@
     <t xml:space="preserve">الأدوات المسموحة</t>
   </si>
   <si>
-    <t xml:space="preserve">أسهم سعودية متوافقة شرعياً (8 أسهم معتمدة من مجلس الإدارة)</t>
+    <t xml:space="preserve">أسهم سعودية متوافقة شرعياً (8 أسهم)</t>
   </si>
   <si>
     <t xml:space="preserve">طلب المتبرع + تنويع مصدر الدخل</t>
@@ -2602,11 +2602,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="97491667"/>
-        <c:axId val="36363071"/>
+        <c:axId val="88347056"/>
+        <c:axId val="23675612"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="97491667"/>
+        <c:axId val="88347056"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2638,7 +2638,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36363071"/>
+        <c:crossAx val="23675612"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2646,7 +2646,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36363071"/>
+        <c:axId val="23675612"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2688,7 +2688,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97491667"/>
+        <c:crossAx val="88347056"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4987,18 +4987,18 @@
         <v>103</v>
       </c>
       <c r="Q25" s="35" t="s">
-        <v>104</v>
+        <v>200</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E26" s="13" t="n">
         <v>141.3</v>
@@ -5011,7 +5011,7 @@
         <v>0.0283085633404105</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I26" s="9" t="s">
         <v>141</v>
@@ -5020,7 +5020,7 @@
         <v>101</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L26" s="9" t="s">
         <v>83</v>
@@ -5038,15 +5038,15 @@
         <v>103</v>
       </c>
       <c r="Q26" s="32" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D27" s="17" t="s">
         <v>40</v>
@@ -5062,16 +5062,16 @@
         <v>0.0341619887730553</v>
       </c>
       <c r="H27" s="17" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I27" s="17" t="s">
         <v>149</v>
       </c>
       <c r="J27" s="17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="K27" s="17" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="L27" s="17" t="s">
         <v>83</v>
@@ -5086,21 +5086,21 @@
         <v>3</v>
       </c>
       <c r="P27" s="39" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="Q27" s="35" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E28" s="13" t="n">
         <v>43.5</v>
@@ -5113,7 +5113,7 @@
         <v>0.0264367816091954</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I28" s="9" t="s">
         <v>141</v>
@@ -5122,7 +5122,7 @@
         <v>154</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="L28" s="9" t="s">
         <v>83</v>
@@ -5140,18 +5140,18 @@
         <v>103</v>
       </c>
       <c r="Q28" s="32" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="18" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E29" s="21" t="n">
         <v>6.65</v>
@@ -5164,16 +5164,16 @@
         <v>0.083609022556391</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I29" s="17" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J29" s="17" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K29" s="17" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="L29" s="17" t="s">
         <v>83</v>
@@ -5188,21 +5188,21 @@
         <v>2</v>
       </c>
       <c r="P29" s="36" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="Q29" s="35" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E30" s="13" t="n">
         <v>8.31</v>
@@ -5215,13 +5215,13 @@
         <v>0.0962695547533093</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K30" s="9" t="s">
         <v>141</v>
@@ -5242,18 +5242,18 @@
         <v>103</v>
       </c>
       <c r="Q30" s="32" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="18" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E31" s="21" t="n">
         <v>7.79</v>
@@ -5266,13 +5266,13 @@
         <v>0.0693196405648267</v>
       </c>
       <c r="H31" s="17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I31" s="17" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J31" s="17" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K31" s="17" t="s">
         <v>141</v>
@@ -5293,18 +5293,18 @@
         <v>103</v>
       </c>
       <c r="Q31" s="35" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E32" s="13" t="n">
         <v>4.31</v>
@@ -5317,13 +5317,13 @@
         <v>0.074245939675174</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I32" s="9" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K32" s="9" t="s">
         <v>141</v>
@@ -5344,18 +5344,18 @@
         <v>103</v>
       </c>
       <c r="Q32" s="32" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="18" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E33" s="21" t="n">
         <v>4.47</v>
@@ -5368,10 +5368,10 @@
         <v>0.0782997762863535</v>
       </c>
       <c r="H33" s="17" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="I33" s="17" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J33" s="17" t="s">
         <v>141</v>
@@ -5395,7 +5395,7 @@
         <v>103</v>
       </c>
       <c r="Q33" s="35" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -5438,7 +5438,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -5450,7 +5450,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -5465,25 +5465,25 @@
         <v>8</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5491,10 +5491,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E6" s="40" t="n">
         <v>46308</v>
@@ -5503,13 +5503,13 @@
         <v>46315</v>
       </c>
       <c r="G6" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="I6" s="16" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5517,10 +5517,10 @@
         <v>2</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E7" s="42" t="n">
         <v>46308</v>
@@ -5529,13 +5529,13 @@
         <v>46317</v>
       </c>
       <c r="G7" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="I7" s="24" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5543,10 +5543,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E8" s="40" t="n">
         <v>46309</v>
@@ -5555,13 +5555,13 @@
         <v>46320</v>
       </c>
       <c r="G8" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5569,10 +5569,10 @@
         <v>4</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
       <c r="E9" s="42" t="n">
         <v>46315</v>
@@ -5581,7 +5581,7 @@
         <v>46341</v>
       </c>
       <c r="G9" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H9" s="17" t="s">
         <v>275</v>
@@ -5607,7 +5607,7 @@
         <v>46328</v>
       </c>
       <c r="G10" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>279</v>
@@ -5633,7 +5633,7 @@
         <v>46338</v>
       </c>
       <c r="G11" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H11" s="17" t="s">
         <v>283</v>
@@ -5659,7 +5659,7 @@
         <v>46371</v>
       </c>
       <c r="G12" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>279</v>
@@ -5676,7 +5676,7 @@
         <v>287</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E13" s="42" t="n">
         <v>46402</v>
@@ -5685,7 +5685,7 @@
         <v>46418</v>
       </c>
       <c r="G13" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H13" s="17" t="s">
         <v>288</v>
@@ -5711,7 +5711,7 @@
         <v>46477</v>
       </c>
       <c r="G14" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>292</v>
@@ -5737,7 +5737,7 @@
         <v>46507</v>
       </c>
       <c r="G15" s="41" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H15" s="17" t="s">
         <v>296</v>

</xml_diff>